<commit_message>
fix: fix PESTLE display error, categorize MBB as bank correctly, enable quarterly fetch, and refine banking valuation with dynamic shares
</commit_message>
<xml_diff>
--- a/Bao cao/MBB/MBB_Model_2026-06.xlsx
+++ b/Bao cao/MBB/MBB_Model_2026-06.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.125</v>
+        <v>0.112</v>
       </c>
     </row>
     <row r="3">
@@ -676,13 +676,13 @@
         <v>3325</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>6916.232051514553</v>
+        <v>4293.129818359497</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>7962.194754753581</v>
+        <v>4942.392832775567</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>9179.314649495553</v>
+        <v>5697.898673776243</v>
       </c>
     </row>
     <row r="5">

</xml_diff>